<commit_message>
added costs to equipment
</commit_message>
<xml_diff>
--- a/equipment_cards.xlsx
+++ b/equipment_cards.xlsx
@@ -16,7 +16,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="55" uniqueCount="55">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="72" uniqueCount="72">
   <si>
     <t>IMAGE</t>
   </si>
@@ -39,13 +39,19 @@
     <t xml:space="preserve">+1 Hand Size. (something else card related)</t>
   </si>
   <si>
+    <t xml:space="preserve">1g, 1k</t>
+  </si>
+  <si>
     <t>cardimages/kaoms_heart.png</t>
   </si>
   <si>
     <t xml:space="preserve">Kaom’s Heart</t>
   </si>
   <si>
-    <t xml:space="preserve">Regenerate 2 Health at the start of every day. +4 Max Health.</t>
+    <t xml:space="preserve">Regenerate 3 Health at the start of every day.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2r, 2g</t>
   </si>
   <si>
     <t>cardimages/whetstone.png</t>
@@ -57,6 +63,9 @@
     <t xml:space="preserve">Deal X+1 damage whenever you deal damage.</t>
   </si>
   <si>
+    <t xml:space="preserve">2r, 1k, 1l</t>
+  </si>
+  <si>
     <t>cardimages/gardeners_bag.png</t>
   </si>
   <si>
@@ -66,6 +75,9 @@
     <t xml:space="preserve">If you gather 3 or more this turn, Prevent 3.</t>
   </si>
   <si>
+    <t xml:space="preserve">1k, 2l</t>
+  </si>
+  <si>
     <t>cardimages/blood_bag.png</t>
   </si>
   <si>
@@ -75,6 +87,9 @@
     <t xml:space="preserve">If total damage dealt this turn is 5 or higher: Draw 2.</t>
   </si>
   <si>
+    <t>1g,1k,1l</t>
+  </si>
+  <si>
     <t>cardimages/spacial_pocket.png</t>
   </si>
   <si>
@@ -84,6 +99,9 @@
     <t xml:space="preserve">Your backpack can hold 5 additional resources.</t>
   </si>
   <si>
+    <t>1g,1k</t>
+  </si>
+  <si>
     <t>cardimages/slingshot.png</t>
   </si>
   <si>
@@ -93,6 +111,9 @@
     <t xml:space="preserve">When you gather you may discard a resource and deal 1 damage.</t>
   </si>
   <si>
+    <t>1r,1l</t>
+  </si>
+  <si>
     <t>cardimages/bfa.png</t>
   </si>
   <si>
@@ -102,13 +123,19 @@
     <t xml:space="preserve">Decrease backpack space by 3. Deal X+1 damage whenever you deal damage.</t>
   </si>
   <si>
+    <t xml:space="preserve">1r, 1g, 1l</t>
+  </si>
+  <si>
     <t>cardimages/tricorn.png</t>
   </si>
   <si>
     <t>Tricorn</t>
   </si>
   <si>
-    <t xml:space="preserve">You may discard and draw 1 new card on the first turn of the day.</t>
+    <t xml:space="preserve">Discard 1 then Draw 1 once per day between turns.</t>
+  </si>
+  <si>
+    <t>2g</t>
   </si>
   <si>
     <t>cardimages/all_seeing_orb.png</t>
@@ -120,13 +147,19 @@
     <t xml:space="preserve">Scry 2 at the start of the day.</t>
   </si>
   <si>
+    <t>2k,1l</t>
+  </si>
+  <si>
     <t>cardimages/day_cycle.png</t>
   </si>
   <si>
     <t xml:space="preserve">Day Cycle</t>
   </si>
   <si>
-    <t xml:space="preserve">Beginning of the day discard X cards and draw X−1 cards.</t>
+    <t xml:space="preserve">Beginning of the day discard X cards and draw X cards.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2k, 2l</t>
   </si>
   <si>
     <t>cardimages/alchemy_orb.png</t>
@@ -138,6 +171,9 @@
     <t xml:space="preserve">Trade any 2 resources for any other resource.</t>
   </si>
   <si>
+    <t>1r,1k,1l</t>
+  </si>
+  <si>
     <t>cardimages/midas_locket.png</t>
   </si>
   <si>
@@ -147,6 +183,9 @@
     <t xml:space="preserve">Spend 1 gold to regenerate 1 health at the start of the day.</t>
   </si>
   <si>
+    <t>1g,2k</t>
+  </si>
+  <si>
     <t>cardimages/seniors_locket.png</t>
   </si>
   <si>
@@ -156,6 +195,9 @@
     <t xml:space="preserve">Burn a resource to play an additional card once per day.</t>
   </si>
   <si>
+    <t>1g,1l,1k</t>
+  </si>
+  <si>
     <t>cardimages/armour_kit.png</t>
   </si>
   <si>
@@ -165,6 +207,9 @@
     <t xml:space="preserve">Your prevent cards prevent X+1 instead.</t>
   </si>
   <si>
+    <t>1r,1g,1l</t>
+  </si>
+  <si>
     <t>cardimages/wooden_shield.png</t>
   </si>
   <si>
@@ -174,6 +219,9 @@
     <t xml:space="preserve">Prevent 2 once per day at any time.</t>
   </si>
   <si>
+    <t>1r,1g</t>
+  </si>
+  <si>
     <t>cardimages/the_hound.png</t>
   </si>
   <si>
@@ -181,6 +229,9 @@
   </si>
   <si>
     <t xml:space="preserve">Scry 1 after you discard a card.</t>
+  </si>
+  <si>
+    <t>2r,1g</t>
   </si>
 </sst>
 </file>
@@ -719,6 +770,7 @@
     <col customWidth="1" min="1" max="1" width="53.421875"/>
     <col customWidth="1" min="2" max="2" width="40.421875"/>
     <col customWidth="1" min="3" max="3" width="82.57421875"/>
+    <col customWidth="1" min="4" max="4" width="12.28125"/>
   </cols>
   <sheetData>
     <row r="1" ht="13.5" customHeight="1">
@@ -745,181 +797,232 @@
       <c r="C2" t="s">
         <v>6</v>
       </c>
+      <c r="D2" t="s">
+        <v>7</v>
+      </c>
     </row>
     <row r="3" ht="21" customHeight="1">
       <c r="A3" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="B3" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="C3" t="s">
-        <v>9</v>
+        <v>10</v>
+      </c>
+      <c r="D3" t="s">
+        <v>11</v>
       </c>
     </row>
     <row r="4" ht="24" customHeight="1">
       <c r="A4" t="s">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="B4" t="s">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="C4" t="s">
-        <v>12</v>
+        <v>14</v>
+      </c>
+      <c r="D4" t="s">
+        <v>15</v>
       </c>
     </row>
     <row r="5" ht="15">
       <c r="A5" t="s">
-        <v>13</v>
+        <v>16</v>
       </c>
       <c r="B5" t="s">
-        <v>14</v>
+        <v>17</v>
       </c>
       <c r="C5" t="s">
-        <v>15</v>
+        <v>18</v>
+      </c>
+      <c r="D5" t="s">
+        <v>19</v>
       </c>
     </row>
     <row r="6" ht="15">
       <c r="A6" t="s">
-        <v>16</v>
+        <v>20</v>
       </c>
       <c r="B6" t="s">
-        <v>17</v>
+        <v>21</v>
       </c>
       <c r="C6" t="s">
-        <v>18</v>
+        <v>22</v>
+      </c>
+      <c r="D6" t="s">
+        <v>23</v>
       </c>
     </row>
     <row r="7" ht="15">
       <c r="A7" t="s">
-        <v>19</v>
+        <v>24</v>
       </c>
       <c r="B7" t="s">
-        <v>20</v>
+        <v>25</v>
       </c>
       <c r="C7" t="s">
-        <v>21</v>
+        <v>26</v>
+      </c>
+      <c r="D7" t="s">
+        <v>27</v>
       </c>
     </row>
     <row r="8" ht="15">
       <c r="A8" t="s">
-        <v>22</v>
+        <v>28</v>
       </c>
       <c r="B8" t="s">
-        <v>23</v>
+        <v>29</v>
       </c>
       <c r="C8" t="s">
-        <v>24</v>
+        <v>30</v>
+      </c>
+      <c r="D8" t="s">
+        <v>31</v>
       </c>
     </row>
     <row r="9" ht="15">
       <c r="A9" t="s">
-        <v>25</v>
+        <v>32</v>
       </c>
       <c r="B9" t="s">
-        <v>26</v>
+        <v>33</v>
       </c>
       <c r="C9" t="s">
-        <v>27</v>
+        <v>34</v>
+      </c>
+      <c r="D9" t="s">
+        <v>35</v>
       </c>
     </row>
     <row r="10" ht="15">
       <c r="A10" t="s">
-        <v>28</v>
+        <v>36</v>
       </c>
       <c r="B10" t="s">
-        <v>29</v>
+        <v>37</v>
       </c>
       <c r="C10" t="s">
-        <v>30</v>
+        <v>38</v>
+      </c>
+      <c r="D10" t="s">
+        <v>39</v>
       </c>
     </row>
     <row r="11" ht="15">
       <c r="A11" t="s">
-        <v>31</v>
+        <v>40</v>
       </c>
       <c r="B11" t="s">
-        <v>32</v>
+        <v>41</v>
       </c>
       <c r="C11" t="s">
-        <v>33</v>
+        <v>42</v>
+      </c>
+      <c r="D11" t="s">
+        <v>43</v>
       </c>
     </row>
     <row r="12" ht="15">
       <c r="A12" t="s">
-        <v>34</v>
+        <v>44</v>
       </c>
       <c r="B12" t="s">
-        <v>35</v>
+        <v>45</v>
       </c>
       <c r="C12" t="s">
-        <v>36</v>
+        <v>46</v>
+      </c>
+      <c r="D12" t="s">
+        <v>47</v>
       </c>
     </row>
     <row r="13" ht="15">
       <c r="A13" t="s">
-        <v>37</v>
+        <v>48</v>
       </c>
       <c r="B13" t="s">
-        <v>38</v>
+        <v>49</v>
       </c>
       <c r="C13" t="s">
-        <v>39</v>
+        <v>50</v>
+      </c>
+      <c r="D13" t="s">
+        <v>51</v>
       </c>
     </row>
     <row r="14" ht="15">
       <c r="A14" t="s">
-        <v>40</v>
+        <v>52</v>
       </c>
       <c r="B14" t="s">
-        <v>41</v>
+        <v>53</v>
       </c>
       <c r="C14" t="s">
-        <v>42</v>
+        <v>54</v>
+      </c>
+      <c r="D14" t="s">
+        <v>55</v>
       </c>
     </row>
     <row r="15" ht="15">
       <c r="A15" t="s">
-        <v>43</v>
+        <v>56</v>
       </c>
       <c r="B15" t="s">
-        <v>44</v>
+        <v>57</v>
       </c>
       <c r="C15" t="s">
-        <v>45</v>
+        <v>58</v>
+      </c>
+      <c r="D15" t="s">
+        <v>59</v>
       </c>
     </row>
     <row r="16" ht="15">
       <c r="A16" t="s">
-        <v>46</v>
+        <v>60</v>
       </c>
       <c r="B16" t="s">
-        <v>47</v>
+        <v>61</v>
       </c>
       <c r="C16" t="s">
-        <v>48</v>
+        <v>62</v>
+      </c>
+      <c r="D16" t="s">
+        <v>63</v>
       </c>
     </row>
     <row r="17" ht="15">
       <c r="A17" t="s">
-        <v>49</v>
+        <v>64</v>
       </c>
       <c r="B17" t="s">
-        <v>50</v>
+        <v>65</v>
       </c>
       <c r="C17" t="s">
-        <v>51</v>
+        <v>66</v>
+      </c>
+      <c r="D17" t="s">
+        <v>67</v>
       </c>
     </row>
     <row r="18" ht="15">
       <c r="A18" t="s">
-        <v>52</v>
+        <v>68</v>
       </c>
       <c r="B18" t="s">
-        <v>53</v>
+        <v>69</v>
       </c>
       <c r="C18" t="s">
-        <v>54</v>
+        <v>70</v>
+      </c>
+      <c r="D18" t="s">
+        <v>71</v>
       </c>
     </row>
   </sheetData>

</xml_diff>